<commit_message>
qualitative A + sottocampioni B (non mi convincono)
</commit_message>
<xml_diff>
--- a/analisi_preliminare_campione_sardi.xlsx
+++ b/analisi_preliminare_campione_sardi.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\salva\Desktop\Code\questionari2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41677A48-538A-425D-A357-52E7C975AD07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28B7326B-A42E-491A-9F32-67EDD13650B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-30" windowWidth="38640" windowHeight="21840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -399,8 +399,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -428,8 +436,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -734,12 +743,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H206"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="9.140625" style="1"/>
+    <col min="5" max="5" width="9.140625" style="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" t="s">
@@ -748,7 +761,7 @@
       <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="F1" t="s">
@@ -761,18 +774,18 @@
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B3" t="s">
+      <c r="B3" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C3">
         <v>1015</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="1" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E4" t="s">
+      <c r="E4" s="1" t="s">
         <v>118</v>
       </c>
     </row>
@@ -785,7 +798,7 @@
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B11" t="s">
+      <c r="B11" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C11">
@@ -796,7 +809,7 @@
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B12" t="s">
+      <c r="B12" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C12">
@@ -807,7 +820,7 @@
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B13" t="s">
+      <c r="B13" s="1" t="s">
         <v>11</v>
       </c>
       <c r="C13">
@@ -818,7 +831,7 @@
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B14" t="s">
+      <c r="B14" s="1" t="s">
         <v>12</v>
       </c>
       <c r="C14">
@@ -829,7 +842,7 @@
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B15" t="s">
+      <c r="B15" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C15">
@@ -840,7 +853,7 @@
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B16" t="s">
+      <c r="B16" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C16">
@@ -851,7 +864,7 @@
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B17" t="s">
+      <c r="B17" s="1" t="s">
         <v>15</v>
       </c>
       <c r="C17">
@@ -862,7 +875,7 @@
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B18" t="s">
+      <c r="B18" s="1" t="s">
         <v>16</v>
       </c>
       <c r="C18">
@@ -873,7 +886,7 @@
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B19" t="s">
+      <c r="B19" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C19">
@@ -884,7 +897,7 @@
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B20" t="s">
+      <c r="B20" s="1" t="s">
         <v>18</v>
       </c>
       <c r="C20">
@@ -895,7 +908,7 @@
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B21" t="s">
+      <c r="B21" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C21">
@@ -906,7 +919,7 @@
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B22" t="s">
+      <c r="B22" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C22">
@@ -917,7 +930,7 @@
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B23" t="s">
+      <c r="B23" s="1" t="s">
         <v>21</v>
       </c>
       <c r="C23">
@@ -933,7 +946,7 @@
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B27" t="s">
+      <c r="B27" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C27">
@@ -942,7 +955,7 @@
       <c r="D27">
         <v>20.7882</v>
       </c>
-      <c r="E27">
+      <c r="E27" s="1">
         <v>727</v>
       </c>
       <c r="F27">
@@ -950,7 +963,7 @@
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B28" t="s">
+      <c r="B28" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C28">
@@ -959,7 +972,7 @@
       <c r="D28">
         <v>10.1478</v>
       </c>
-      <c r="E28">
+      <c r="E28" s="1">
         <v>505</v>
       </c>
       <c r="F28">
@@ -967,7 +980,7 @@
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B29" t="s">
+      <c r="B29" s="1" t="s">
         <v>23</v>
       </c>
       <c r="C29">
@@ -976,7 +989,7 @@
       <c r="D29">
         <v>6.4039000000000001</v>
       </c>
-      <c r="E29">
+      <c r="E29" s="1">
         <v>141</v>
       </c>
       <c r="F29">
@@ -984,7 +997,7 @@
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B30" t="s">
+      <c r="B30" s="1" t="s">
         <v>11</v>
       </c>
       <c r="C30">
@@ -993,7 +1006,7 @@
       <c r="D30">
         <v>6.0099</v>
       </c>
-      <c r="E30">
+      <c r="E30" s="1">
         <v>168</v>
       </c>
       <c r="F30">
@@ -1001,7 +1014,7 @@
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B31" t="s">
+      <c r="B31" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C31">
@@ -1010,7 +1023,7 @@
       <c r="D31">
         <v>4.6304999999999996</v>
       </c>
-      <c r="E31">
+      <c r="E31" s="1">
         <v>188</v>
       </c>
       <c r="F31">
@@ -1018,7 +1031,7 @@
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B32" t="s">
+      <c r="B32" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C32">
@@ -1027,7 +1040,7 @@
       <c r="D32">
         <v>4.532</v>
       </c>
-      <c r="E32">
+      <c r="E32" s="1">
         <v>110</v>
       </c>
       <c r="F32">
@@ -1035,7 +1048,7 @@
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B33" t="s">
+      <c r="B33" s="1" t="s">
         <v>12</v>
       </c>
       <c r="C33">
@@ -1044,7 +1057,7 @@
       <c r="D33">
         <v>4.0393999999999997</v>
       </c>
-      <c r="E33">
+      <c r="E33" s="1">
         <v>102</v>
       </c>
       <c r="F33">
@@ -1052,7 +1065,7 @@
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B34" t="s">
+      <c r="B34" s="1" t="s">
         <v>15</v>
       </c>
       <c r="C34">
@@ -1061,7 +1074,7 @@
       <c r="D34">
         <v>0.98519999999999996</v>
       </c>
-      <c r="E34">
+      <c r="E34" s="1">
         <v>17</v>
       </c>
       <c r="F34">
@@ -1069,7 +1082,7 @@
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B35" t="s">
+      <c r="B35" s="1" t="s">
         <v>24</v>
       </c>
       <c r="C35">
@@ -1078,7 +1091,7 @@
       <c r="D35">
         <v>0.88670000000000004</v>
       </c>
-      <c r="E35">
+      <c r="E35" s="1">
         <v>12</v>
       </c>
       <c r="F35">
@@ -1086,7 +1099,7 @@
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B36" t="s">
+      <c r="B36" s="1" t="s">
         <v>16</v>
       </c>
       <c r="C36">
@@ -1095,7 +1108,7 @@
       <c r="D36">
         <v>0.68969999999999998</v>
       </c>
-      <c r="E36">
+      <c r="E36" s="1">
         <v>17</v>
       </c>
       <c r="F36">
@@ -1103,7 +1116,7 @@
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B37" t="s">
+      <c r="B37" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C37">
@@ -1112,7 +1125,7 @@
       <c r="D37">
         <v>0.49259999999999998</v>
       </c>
-      <c r="E37">
+      <c r="E37" s="1">
         <v>14</v>
       </c>
       <c r="F37">
@@ -1120,7 +1133,7 @@
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B38" t="s">
+      <c r="B38" s="1" t="s">
         <v>25</v>
       </c>
       <c r="C38">
@@ -1129,7 +1142,7 @@
       <c r="D38">
         <v>0.49259999999999998</v>
       </c>
-      <c r="E38">
+      <c r="E38" s="1">
         <v>30</v>
       </c>
       <c r="F38">
@@ -1137,7 +1150,7 @@
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B39" t="s">
+      <c r="B39" s="1" t="s">
         <v>26</v>
       </c>
       <c r="C39">
@@ -1146,7 +1159,7 @@
       <c r="D39">
         <v>0.39410000000000001</v>
       </c>
-      <c r="E39">
+      <c r="E39" s="1">
         <v>25</v>
       </c>
       <c r="F39">
@@ -1154,7 +1167,7 @@
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B40" t="s">
+      <c r="B40" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C40">
@@ -1163,7 +1176,7 @@
       <c r="D40">
         <v>0.19700000000000001</v>
       </c>
-      <c r="E40">
+      <c r="E40" s="1">
         <v>7</v>
       </c>
       <c r="F40">
@@ -1171,7 +1184,7 @@
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B41" t="s">
+      <c r="B41" s="1" t="s">
         <v>27</v>
       </c>
       <c r="C41">
@@ -1180,7 +1193,7 @@
       <c r="D41">
         <v>0.19700000000000001</v>
       </c>
-      <c r="E41">
+      <c r="E41" s="1">
         <v>8</v>
       </c>
       <c r="F41">
@@ -1188,7 +1201,7 @@
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B42" t="s">
+      <c r="B42" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C42">
@@ -1197,7 +1210,7 @@
       <c r="D42">
         <v>9.8500000000000004E-2</v>
       </c>
-      <c r="E42">
+      <c r="E42" s="1">
         <v>2</v>
       </c>
       <c r="F42">
@@ -1205,7 +1218,7 @@
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B43" t="s">
+      <c r="B43" s="1" t="s">
         <v>28</v>
       </c>
       <c r="C43">
@@ -1214,7 +1227,7 @@
       <c r="D43">
         <v>9.8500000000000004E-2</v>
       </c>
-      <c r="E43">
+      <c r="E43" s="1">
         <v>1</v>
       </c>
       <c r="F43">
@@ -1222,7 +1235,7 @@
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B44" t="s">
+      <c r="B44" s="1" t="s">
         <v>21</v>
       </c>
       <c r="C44">
@@ -1231,7 +1244,7 @@
       <c r="D44">
         <v>9.8500000000000004E-2</v>
       </c>
-      <c r="E44">
+      <c r="E44" s="1">
         <v>2</v>
       </c>
       <c r="F44">
@@ -1244,7 +1257,7 @@
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B48" t="s">
+      <c r="B48" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C48">
@@ -1253,7 +1266,7 @@
       <c r="D48">
         <v>38.817700000000002</v>
       </c>
-      <c r="E48">
+      <c r="E48" s="1">
         <v>216</v>
       </c>
       <c r="F48">
@@ -1264,7 +1277,7 @@
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B49" t="s">
+      <c r="B49" s="1" t="s">
         <v>31</v>
       </c>
       <c r="C49">
@@ -1273,7 +1286,7 @@
       <c r="D49">
         <v>23.940899999999999</v>
       </c>
-      <c r="E49">
+      <c r="E49" s="1">
         <v>855</v>
       </c>
       <c r="F49">
@@ -1281,7 +1294,7 @@
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B50" t="s">
+      <c r="B50" s="1" t="s">
         <v>32</v>
       </c>
       <c r="C50">
@@ -1290,7 +1303,7 @@
       <c r="D50">
         <v>21.0837</v>
       </c>
-      <c r="E50">
+      <c r="E50" s="1">
         <v>724</v>
       </c>
       <c r="F50">
@@ -1298,7 +1311,7 @@
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B51" t="s">
+      <c r="B51" s="1" t="s">
         <v>33</v>
       </c>
       <c r="C51">
@@ -1307,7 +1320,7 @@
       <c r="D51">
         <v>16.157599999999999</v>
       </c>
-      <c r="E51">
+      <c r="E51" s="1">
         <v>497</v>
       </c>
       <c r="F51">
@@ -1320,7 +1333,7 @@
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B55" t="s">
+      <c r="B55" s="1" t="s">
         <v>35</v>
       </c>
       <c r="C55">
@@ -1329,7 +1342,7 @@
       <c r="D55">
         <v>15.0739</v>
       </c>
-      <c r="E55">
+      <c r="E55" s="1">
         <v>502</v>
       </c>
       <c r="F55">
@@ -1337,7 +1350,7 @@
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B56" t="s">
+      <c r="B56" s="1" t="s">
         <v>36</v>
       </c>
       <c r="C56">
@@ -1346,7 +1359,7 @@
       <c r="D56">
         <v>13.004899999999999</v>
       </c>
-      <c r="E56">
+      <c r="E56" s="1">
         <v>361</v>
       </c>
       <c r="F56">
@@ -1354,7 +1367,7 @@
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B57" t="s">
+      <c r="B57" s="1" t="s">
         <v>37</v>
       </c>
       <c r="C57">
@@ -1363,7 +1376,7 @@
       <c r="D57">
         <v>10.738899999999999</v>
       </c>
-      <c r="E57">
+      <c r="E57" s="1">
         <v>332</v>
       </c>
       <c r="F57">
@@ -1371,7 +1384,7 @@
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B58" t="s">
+      <c r="B58" s="1" t="s">
         <v>38</v>
       </c>
       <c r="C58">
@@ -1380,7 +1393,7 @@
       <c r="D58">
         <v>9.7537000000000003</v>
       </c>
-      <c r="E58">
+      <c r="E58" s="1">
         <v>264</v>
       </c>
       <c r="F58">
@@ -1388,7 +1401,7 @@
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B59" t="s">
+      <c r="B59" s="1" t="s">
         <v>39</v>
       </c>
       <c r="C59">
@@ -1397,7 +1410,7 @@
       <c r="D59">
         <v>7.0936000000000003</v>
       </c>
-      <c r="E59">
+      <c r="E59" s="1">
         <v>285</v>
       </c>
       <c r="F59">
@@ -1405,7 +1418,7 @@
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B60" t="s">
+      <c r="B60" s="1" t="s">
         <v>40</v>
       </c>
       <c r="C60">
@@ -1414,7 +1427,7 @@
       <c r="D60">
         <v>5.5171999999999999</v>
       </c>
-      <c r="E60">
+      <c r="E60" s="1">
         <v>332</v>
       </c>
       <c r="F60">
@@ -1430,7 +1443,7 @@
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B64" t="s">
+      <c r="B64" s="1" t="s">
         <v>40</v>
       </c>
       <c r="C64">
@@ -1441,7 +1454,7 @@
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B65" t="s">
+      <c r="B65" s="1" t="s">
         <v>35</v>
       </c>
       <c r="C65">
@@ -1452,7 +1465,7 @@
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B66" t="s">
+      <c r="B66" s="1" t="s">
         <v>38</v>
       </c>
       <c r="C66">
@@ -1463,7 +1476,7 @@
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B67" t="s">
+      <c r="B67" s="1" t="s">
         <v>36</v>
       </c>
       <c r="C67">
@@ -1474,7 +1487,7 @@
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B68" t="s">
+      <c r="B68" s="1" t="s">
         <v>37</v>
       </c>
       <c r="C68">
@@ -1485,7 +1498,7 @@
       </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B69" t="s">
+      <c r="B69" s="1" t="s">
         <v>39</v>
       </c>
       <c r="C69">
@@ -1504,7 +1517,7 @@
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B73" t="s">
+      <c r="B73" s="1" t="s">
         <v>43</v>
       </c>
       <c r="C73">
@@ -1515,7 +1528,7 @@
       </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B74" t="s">
+      <c r="B74" s="1" t="s">
         <v>44</v>
       </c>
       <c r="C74">
@@ -1526,7 +1539,7 @@
       </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B75" t="s">
+      <c r="B75" s="1" t="s">
         <v>45</v>
       </c>
       <c r="C75">
@@ -1537,7 +1550,7 @@
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B76" t="s">
+      <c r="B76" s="1" t="s">
         <v>46</v>
       </c>
       <c r="C76">
@@ -1548,7 +1561,7 @@
       </c>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B77" t="s">
+      <c r="B77" s="1" t="s">
         <v>47</v>
       </c>
       <c r="C77">
@@ -1564,7 +1577,7 @@
       </c>
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B81" t="s">
+      <c r="B81" s="1" t="s">
         <v>45</v>
       </c>
       <c r="C81">
@@ -1573,7 +1586,7 @@
       <c r="D81">
         <v>17.931000000000001</v>
       </c>
-      <c r="E81">
+      <c r="E81" s="1">
         <v>372</v>
       </c>
       <c r="F81">
@@ -1581,7 +1594,7 @@
       </c>
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B82" t="s">
+      <c r="B82" s="1" t="s">
         <v>46</v>
       </c>
       <c r="C82">
@@ -1590,7 +1603,7 @@
       <c r="D82">
         <v>17.438400000000001</v>
       </c>
-      <c r="E82">
+      <c r="E82" s="1">
         <v>1097</v>
       </c>
       <c r="F82">
@@ -1598,7 +1611,7 @@
       </c>
     </row>
     <row r="83" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B83" t="s">
+      <c r="B83" s="1" t="s">
         <v>47</v>
       </c>
       <c r="C83">
@@ -1607,7 +1620,7 @@
       <c r="D83">
         <v>14.581300000000001</v>
       </c>
-      <c r="E83">
+      <c r="E83" s="1">
         <v>464</v>
       </c>
       <c r="F83">
@@ -1615,7 +1628,7 @@
       </c>
     </row>
     <row r="84" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B84" t="s">
+      <c r="B84" s="1" t="s">
         <v>43</v>
       </c>
       <c r="C84">
@@ -1624,7 +1637,7 @@
       <c r="D84">
         <v>10.936</v>
       </c>
-      <c r="E84">
+      <c r="E84" s="1">
         <v>136</v>
       </c>
       <c r="F84">
@@ -1632,7 +1645,7 @@
       </c>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B85" t="s">
+      <c r="B85" s="1" t="s">
         <v>44</v>
       </c>
       <c r="C85">
@@ -1641,7 +1654,7 @@
       <c r="D85">
         <v>0.29559999999999997</v>
       </c>
-      <c r="E85">
+      <c r="E85" s="1">
         <v>7</v>
       </c>
       <c r="F85">
@@ -1657,7 +1670,7 @@
       </c>
     </row>
     <row r="89" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B89" t="s">
+      <c r="B89" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C89">
@@ -1668,7 +1681,7 @@
       </c>
     </row>
     <row r="90" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B90" t="s">
+      <c r="B90" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C90">
@@ -1679,7 +1692,7 @@
       </c>
     </row>
     <row r="91" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B91" t="s">
+      <c r="B91" s="1" t="s">
         <v>11</v>
       </c>
       <c r="C91">
@@ -1690,7 +1703,7 @@
       </c>
     </row>
     <row r="92" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B92" t="s">
+      <c r="B92" s="1" t="s">
         <v>12</v>
       </c>
       <c r="C92">
@@ -1701,7 +1714,7 @@
       </c>
     </row>
     <row r="93" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B93" t="s">
+      <c r="B93" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C93">
@@ -1712,7 +1725,7 @@
       </c>
     </row>
     <row r="94" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B94" t="s">
+      <c r="B94" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C94">
@@ -1723,7 +1736,7 @@
       </c>
     </row>
     <row r="95" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B95" t="s">
+      <c r="B95" s="1" t="s">
         <v>15</v>
       </c>
       <c r="C95">
@@ -1734,7 +1747,7 @@
       </c>
     </row>
     <row r="96" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B96" t="s">
+      <c r="B96" s="1" t="s">
         <v>50</v>
       </c>
       <c r="C96">
@@ -1745,7 +1758,7 @@
       </c>
     </row>
     <row r="97" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B97" t="s">
+      <c r="B97" s="1" t="s">
         <v>18</v>
       </c>
       <c r="C97">
@@ -1756,7 +1769,7 @@
       </c>
     </row>
     <row r="98" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B98" t="s">
+      <c r="B98" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C98">
@@ -1767,7 +1780,7 @@
       </c>
     </row>
     <row r="99" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B99" t="s">
+      <c r="B99" s="1" t="s">
         <v>16</v>
       </c>
       <c r="C99">
@@ -1778,7 +1791,7 @@
       </c>
     </row>
     <row r="100" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B100" t="s">
+      <c r="B100" s="1" t="s">
         <v>28</v>
       </c>
       <c r="C100">
@@ -1789,7 +1802,7 @@
       </c>
     </row>
     <row r="101" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B101" t="s">
+      <c r="B101" s="1" t="s">
         <v>51</v>
       </c>
       <c r="C101">
@@ -1800,7 +1813,7 @@
       </c>
     </row>
     <row r="102" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B102" t="s">
+      <c r="B102" s="1" t="s">
         <v>52</v>
       </c>
       <c r="C102">
@@ -1811,7 +1824,7 @@
       </c>
     </row>
     <row r="103" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B103" t="s">
+      <c r="B103" s="1" t="s">
         <v>53</v>
       </c>
       <c r="C103">
@@ -1822,7 +1835,7 @@
       </c>
     </row>
     <row r="104" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B104" t="s">
+      <c r="B104" s="1" t="s">
         <v>54</v>
       </c>
       <c r="C104">
@@ -1833,7 +1846,7 @@
       </c>
     </row>
     <row r="105" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B105" t="s">
+      <c r="B105" s="1" t="s">
         <v>55</v>
       </c>
       <c r="C105">
@@ -1844,7 +1857,7 @@
       </c>
     </row>
     <row r="106" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B106" t="s">
+      <c r="B106" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C106">
@@ -1855,7 +1868,7 @@
       </c>
     </row>
     <row r="107" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B107" t="s">
+      <c r="B107" s="1" t="s">
         <v>56</v>
       </c>
       <c r="C107">
@@ -1866,7 +1879,7 @@
       </c>
     </row>
     <row r="108" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B108" t="s">
+      <c r="B108" s="1" t="s">
         <v>57</v>
       </c>
       <c r="C108">
@@ -1877,7 +1890,7 @@
       </c>
     </row>
     <row r="109" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B109" t="s">
+      <c r="B109" s="1" t="s">
         <v>58</v>
       </c>
       <c r="C109">
@@ -1888,7 +1901,7 @@
       </c>
     </row>
     <row r="110" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B110" t="s">
+      <c r="B110" s="1" t="s">
         <v>59</v>
       </c>
       <c r="C110">
@@ -1899,7 +1912,7 @@
       </c>
     </row>
     <row r="111" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B111" t="s">
+      <c r="B111" s="1" t="s">
         <v>60</v>
       </c>
       <c r="C111">
@@ -1910,7 +1923,7 @@
       </c>
     </row>
     <row r="112" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B112" t="s">
+      <c r="B112" s="1" t="s">
         <v>61</v>
       </c>
       <c r="C112">
@@ -1921,7 +1934,7 @@
       </c>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B113" t="s">
+      <c r="B113" s="1" t="s">
         <v>62</v>
       </c>
       <c r="C113">
@@ -1932,7 +1945,7 @@
       </c>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B114" t="s">
+      <c r="B114" s="1" t="s">
         <v>63</v>
       </c>
       <c r="C114">
@@ -1943,7 +1956,7 @@
       </c>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B115" t="s">
+      <c r="B115" s="1" t="s">
         <v>64</v>
       </c>
       <c r="C115">
@@ -1954,7 +1967,7 @@
       </c>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B116" t="s">
+      <c r="B116" s="1" t="s">
         <v>65</v>
       </c>
       <c r="C116">
@@ -1965,7 +1978,7 @@
       </c>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B117" t="s">
+      <c r="B117" s="1" t="s">
         <v>66</v>
       </c>
       <c r="C117">
@@ -1976,7 +1989,7 @@
       </c>
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B118" t="s">
+      <c r="B118" s="1" t="s">
         <v>67</v>
       </c>
       <c r="C118">
@@ -1987,7 +2000,7 @@
       </c>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B119" t="s">
+      <c r="B119" s="1" t="s">
         <v>68</v>
       </c>
       <c r="C119">
@@ -1998,7 +2011,7 @@
       </c>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B120" t="s">
+      <c r="B120" s="1" t="s">
         <v>69</v>
       </c>
       <c r="C120">
@@ -2009,7 +2022,7 @@
       </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B121" t="s">
+      <c r="B121" s="1" t="s">
         <v>70</v>
       </c>
       <c r="C121">
@@ -2025,7 +2038,7 @@
       </c>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B125" t="s">
+      <c r="B125" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C125">
@@ -2034,7 +2047,7 @@
       <c r="D125">
         <v>17.931000000000001</v>
       </c>
-      <c r="E125">
+      <c r="E125" s="1">
         <v>615</v>
       </c>
       <c r="F125">
@@ -2042,7 +2055,7 @@
       </c>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B126" t="s">
+      <c r="B126" s="1" t="s">
         <v>11</v>
       </c>
       <c r="C126">
@@ -2051,7 +2064,7 @@
       <c r="D126">
         <v>10.936</v>
       </c>
-      <c r="E126">
+      <c r="E126" s="1">
         <v>272</v>
       </c>
       <c r="F126">
@@ -2059,7 +2072,7 @@
       </c>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B127" t="s">
+      <c r="B127" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C127">
@@ -2068,7 +2081,7 @@
       <c r="D127">
         <v>5.2217000000000002</v>
       </c>
-      <c r="E127">
+      <c r="E127" s="1">
         <v>315</v>
       </c>
       <c r="F127">
@@ -2076,7 +2089,7 @@
       </c>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B128" t="s">
+      <c r="B128" s="1" t="s">
         <v>12</v>
       </c>
       <c r="C128">
@@ -2085,7 +2098,7 @@
       <c r="D128">
         <v>4.335</v>
       </c>
-      <c r="E128">
+      <c r="E128" s="1">
         <v>113</v>
       </c>
       <c r="F128">
@@ -2093,7 +2106,7 @@
       </c>
     </row>
     <row r="129" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B129" t="s">
+      <c r="B129" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C129">
@@ -2102,7 +2115,7 @@
       <c r="D129">
         <v>3.6453000000000002</v>
       </c>
-      <c r="E129">
+      <c r="E129" s="1">
         <v>114</v>
       </c>
       <c r="F129">
@@ -2110,7 +2123,7 @@
       </c>
     </row>
     <row r="130" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B130" t="s">
+      <c r="B130" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C130">
@@ -2119,7 +2132,7 @@
       <c r="D130">
         <v>3.5468000000000002</v>
       </c>
-      <c r="E130">
+      <c r="E130" s="1">
         <v>134</v>
       </c>
       <c r="F130">
@@ -2127,7 +2140,7 @@
       </c>
     </row>
     <row r="131" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B131" t="s">
+      <c r="B131" s="1" t="s">
         <v>23</v>
       </c>
       <c r="C131">
@@ -2136,7 +2149,7 @@
       <c r="D131">
         <v>2.4630999999999998</v>
       </c>
-      <c r="E131">
+      <c r="E131" s="1">
         <v>69</v>
       </c>
       <c r="F131">
@@ -2144,7 +2157,7 @@
       </c>
     </row>
     <row r="132" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B132" t="s">
+      <c r="B132" s="1" t="s">
         <v>26</v>
       </c>
       <c r="C132">
@@ -2153,7 +2166,7 @@
       <c r="D132">
         <v>1.1822999999999999</v>
       </c>
-      <c r="E132">
+      <c r="E132" s="1">
         <v>73</v>
       </c>
       <c r="F132">
@@ -2161,7 +2174,7 @@
       </c>
     </row>
     <row r="133" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B133" t="s">
+      <c r="B133" s="1" t="s">
         <v>15</v>
       </c>
       <c r="C133">
@@ -2170,7 +2183,7 @@
       <c r="D133">
         <v>1.0837000000000001</v>
       </c>
-      <c r="E133">
+      <c r="E133" s="1">
         <v>22</v>
       </c>
       <c r="F133">
@@ -2178,7 +2191,7 @@
       </c>
     </row>
     <row r="134" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B134" t="s">
+      <c r="B134" s="1" t="s">
         <v>24</v>
       </c>
       <c r="C134">
@@ -2187,7 +2200,7 @@
       <c r="D134">
         <v>0.68969999999999998</v>
       </c>
-      <c r="E134">
+      <c r="E134" s="1">
         <v>11</v>
       </c>
       <c r="F134">
@@ -2195,7 +2208,7 @@
       </c>
     </row>
     <row r="135" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B135" t="s">
+      <c r="B135" s="1" t="s">
         <v>18</v>
       </c>
       <c r="C135">
@@ -2204,7 +2217,7 @@
       <c r="D135">
         <v>0.68969999999999998</v>
       </c>
-      <c r="E135">
+      <c r="E135" s="1">
         <v>29</v>
       </c>
       <c r="F135">
@@ -2212,7 +2225,7 @@
       </c>
     </row>
     <row r="136" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B136" t="s">
+      <c r="B136" s="1" t="s">
         <v>16</v>
       </c>
       <c r="C136">
@@ -2221,7 +2234,7 @@
       <c r="D136">
         <v>0.68969999999999998</v>
       </c>
-      <c r="E136">
+      <c r="E136" s="1">
         <v>21</v>
       </c>
       <c r="F136">
@@ -2229,7 +2242,7 @@
       </c>
     </row>
     <row r="137" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B137" t="s">
+      <c r="B137" s="1" t="s">
         <v>54</v>
       </c>
       <c r="C137">
@@ -2238,7 +2251,7 @@
       <c r="D137">
         <v>0.59109999999999996</v>
       </c>
-      <c r="E137">
+      <c r="E137" s="1">
         <v>17</v>
       </c>
       <c r="F137">
@@ -2246,7 +2259,7 @@
       </c>
     </row>
     <row r="138" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B138" t="s">
+      <c r="B138" s="1" t="s">
         <v>51</v>
       </c>
       <c r="C138">
@@ -2255,7 +2268,7 @@
       <c r="D138">
         <v>0.49259999999999998</v>
       </c>
-      <c r="E138">
+      <c r="E138" s="1">
         <v>16</v>
       </c>
       <c r="F138">
@@ -2263,7 +2276,7 @@
       </c>
     </row>
     <row r="139" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B139" t="s">
+      <c r="B139" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C139">
@@ -2272,7 +2285,7 @@
       <c r="D139">
         <v>0.49259999999999998</v>
       </c>
-      <c r="E139">
+      <c r="E139" s="1">
         <v>15</v>
       </c>
       <c r="F139">
@@ -2280,7 +2293,7 @@
       </c>
     </row>
     <row r="140" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B140" t="s">
+      <c r="B140" s="1" t="s">
         <v>72</v>
       </c>
       <c r="C140">
@@ -2289,7 +2302,7 @@
       <c r="D140">
         <v>0.39410000000000001</v>
       </c>
-      <c r="E140">
+      <c r="E140" s="1">
         <v>13</v>
       </c>
       <c r="F140">
@@ -2297,7 +2310,7 @@
       </c>
     </row>
     <row r="141" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B141" t="s">
+      <c r="B141" s="1" t="s">
         <v>25</v>
       </c>
       <c r="C141">
@@ -2306,7 +2319,7 @@
       <c r="D141">
         <v>0.39410000000000001</v>
       </c>
-      <c r="E141">
+      <c r="E141" s="1">
         <v>31</v>
       </c>
       <c r="F141">
@@ -2314,7 +2327,7 @@
       </c>
     </row>
     <row r="142" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B142" t="s">
+      <c r="B142" s="1" t="s">
         <v>53</v>
       </c>
       <c r="C142">
@@ -2323,7 +2336,7 @@
       <c r="D142">
         <v>0.29559999999999997</v>
       </c>
-      <c r="E142">
+      <c r="E142" s="1">
         <v>7</v>
       </c>
       <c r="F142">
@@ -2331,7 +2344,7 @@
       </c>
     </row>
     <row r="143" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B143" t="s">
+      <c r="B143" s="1" t="s">
         <v>66</v>
       </c>
       <c r="C143">
@@ -2340,7 +2353,7 @@
       <c r="D143">
         <v>0.29559999999999997</v>
       </c>
-      <c r="E143">
+      <c r="E143" s="1">
         <v>8</v>
       </c>
       <c r="F143">
@@ -2348,7 +2361,7 @@
       </c>
     </row>
     <row r="144" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B144" t="s">
+      <c r="B144" s="1" t="s">
         <v>67</v>
       </c>
       <c r="C144">
@@ -2357,7 +2370,7 @@
       <c r="D144">
         <v>0.29559999999999997</v>
       </c>
-      <c r="E144">
+      <c r="E144" s="1">
         <v>9</v>
       </c>
       <c r="F144">
@@ -2365,7 +2378,7 @@
       </c>
     </row>
     <row r="145" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B145" t="s">
+      <c r="B145" s="1" t="s">
         <v>28</v>
       </c>
       <c r="C145">
@@ -2374,7 +2387,7 @@
       <c r="D145">
         <v>0.19700000000000001</v>
       </c>
-      <c r="E145">
+      <c r="E145" s="1">
         <v>3</v>
       </c>
       <c r="F145">
@@ -2382,7 +2395,7 @@
       </c>
     </row>
     <row r="146" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B146" t="s">
+      <c r="B146" s="1" t="s">
         <v>73</v>
       </c>
       <c r="C146">
@@ -2391,7 +2404,7 @@
       <c r="D146">
         <v>0.19700000000000001</v>
       </c>
-      <c r="E146">
+      <c r="E146" s="1">
         <v>9</v>
       </c>
       <c r="F146">
@@ -2399,7 +2412,7 @@
       </c>
     </row>
     <row r="147" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B147" t="s">
+      <c r="B147" s="1" t="s">
         <v>50</v>
       </c>
       <c r="C147">
@@ -2408,7 +2421,7 @@
       <c r="D147">
         <v>0.19700000000000001</v>
       </c>
-      <c r="E147">
+      <c r="E147" s="1">
         <v>6</v>
       </c>
       <c r="F147">
@@ -2416,7 +2429,7 @@
       </c>
     </row>
     <row r="148" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B148" t="s">
+      <c r="B148" s="1" t="s">
         <v>74</v>
       </c>
       <c r="C148">
@@ -2425,7 +2438,7 @@
       <c r="D148">
         <v>0.19700000000000001</v>
       </c>
-      <c r="E148">
+      <c r="E148" s="1">
         <v>5</v>
       </c>
       <c r="F148">
@@ -2433,7 +2446,7 @@
       </c>
     </row>
     <row r="149" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B149" t="s">
+      <c r="B149" s="1" t="s">
         <v>75</v>
       </c>
       <c r="C149">
@@ -2442,7 +2455,7 @@
       <c r="D149">
         <v>0.19700000000000001</v>
       </c>
-      <c r="E149">
+      <c r="E149" s="1">
         <v>2</v>
       </c>
       <c r="F149">
@@ -2450,7 +2463,7 @@
       </c>
     </row>
     <row r="150" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B150" t="s">
+      <c r="B150" s="1" t="s">
         <v>76</v>
       </c>
       <c r="C150">
@@ -2459,7 +2472,7 @@
       <c r="D150">
         <v>0.19700000000000001</v>
       </c>
-      <c r="E150">
+      <c r="E150" s="1">
         <v>4</v>
       </c>
       <c r="F150">
@@ -2467,7 +2480,7 @@
       </c>
     </row>
     <row r="151" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B151" t="s">
+      <c r="B151" s="1" t="s">
         <v>52</v>
       </c>
       <c r="C151">
@@ -2476,7 +2489,7 @@
       <c r="D151">
         <v>0.19700000000000001</v>
       </c>
-      <c r="E151">
+      <c r="E151" s="1">
         <v>8</v>
       </c>
       <c r="F151">
@@ -2484,7 +2497,7 @@
       </c>
     </row>
     <row r="152" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B152" t="s">
+      <c r="B152" s="1" t="s">
         <v>77</v>
       </c>
       <c r="C152">
@@ -2493,7 +2506,7 @@
       <c r="D152">
         <v>0.19700000000000001</v>
       </c>
-      <c r="E152">
+      <c r="E152" s="1">
         <v>4</v>
       </c>
       <c r="F152">
@@ -2501,7 +2514,7 @@
       </c>
     </row>
     <row r="153" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B153" t="s">
+      <c r="B153" s="1" t="s">
         <v>65</v>
       </c>
       <c r="C153">
@@ -2510,7 +2523,7 @@
       <c r="D153">
         <v>0.19700000000000001</v>
       </c>
-      <c r="E153">
+      <c r="E153" s="1">
         <v>6</v>
       </c>
       <c r="F153">
@@ -2518,7 +2531,7 @@
       </c>
     </row>
     <row r="154" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B154" t="s">
+      <c r="B154" s="1" t="s">
         <v>27</v>
       </c>
       <c r="C154">
@@ -2527,7 +2540,7 @@
       <c r="D154">
         <v>0.19700000000000001</v>
       </c>
-      <c r="E154">
+      <c r="E154" s="1">
         <v>8</v>
       </c>
       <c r="F154">
@@ -2535,7 +2548,7 @@
       </c>
     </row>
     <row r="155" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B155" t="s">
+      <c r="B155" s="1" t="s">
         <v>78</v>
       </c>
       <c r="C155">
@@ -2544,7 +2557,7 @@
       <c r="D155">
         <v>0.19700000000000001</v>
       </c>
-      <c r="E155">
+      <c r="E155" s="1">
         <v>4</v>
       </c>
       <c r="F155">
@@ -2552,7 +2565,7 @@
       </c>
     </row>
     <row r="156" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B156" t="s">
+      <c r="B156" s="1" t="s">
         <v>79</v>
       </c>
       <c r="C156">
@@ -2561,7 +2574,7 @@
       <c r="D156">
         <v>0.19700000000000001</v>
       </c>
-      <c r="E156">
+      <c r="E156" s="1">
         <v>3</v>
       </c>
       <c r="F156">
@@ -2569,7 +2582,7 @@
       </c>
     </row>
     <row r="157" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B157" t="s">
+      <c r="B157" s="1" t="s">
         <v>70</v>
       </c>
       <c r="C157">
@@ -2578,7 +2591,7 @@
       <c r="D157">
         <v>0.19700000000000001</v>
       </c>
-      <c r="E157">
+      <c r="E157" s="1">
         <v>3</v>
       </c>
       <c r="F157">
@@ -2586,7 +2599,7 @@
       </c>
     </row>
     <row r="158" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B158" t="s">
+      <c r="B158" s="1" t="s">
         <v>80</v>
       </c>
       <c r="C158">
@@ -2595,7 +2608,7 @@
       <c r="D158">
         <v>0.19700000000000001</v>
       </c>
-      <c r="E158">
+      <c r="E158" s="1">
         <v>2</v>
       </c>
       <c r="F158">
@@ -2603,7 +2616,7 @@
       </c>
     </row>
     <row r="159" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B159" t="s">
+      <c r="B159" s="1" t="s">
         <v>81</v>
       </c>
       <c r="C159">
@@ -2612,7 +2625,7 @@
       <c r="D159">
         <v>0.19700000000000001</v>
       </c>
-      <c r="E159">
+      <c r="E159" s="1">
         <v>6</v>
       </c>
       <c r="F159">
@@ -2620,7 +2633,7 @@
       </c>
     </row>
     <row r="160" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B160" t="s">
+      <c r="B160" s="1" t="s">
         <v>82</v>
       </c>
       <c r="C160">
@@ -2629,7 +2642,7 @@
       <c r="D160">
         <v>9.8500000000000004E-2</v>
       </c>
-      <c r="E160">
+      <c r="E160" s="1">
         <v>5</v>
       </c>
       <c r="F160">
@@ -2637,7 +2650,7 @@
       </c>
     </row>
     <row r="161" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B161" t="s">
+      <c r="B161" s="1" t="s">
         <v>83</v>
       </c>
       <c r="C161">
@@ -2646,7 +2659,7 @@
       <c r="D161">
         <v>9.8500000000000004E-2</v>
       </c>
-      <c r="E161">
+      <c r="E161" s="1">
         <v>2</v>
       </c>
       <c r="F161">
@@ -2654,7 +2667,7 @@
       </c>
     </row>
     <row r="162" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B162" t="s">
+      <c r="B162" s="1" t="s">
         <v>84</v>
       </c>
       <c r="C162">
@@ -2663,7 +2676,7 @@
       <c r="D162">
         <v>9.8500000000000004E-2</v>
       </c>
-      <c r="E162">
+      <c r="E162" s="1">
         <v>2</v>
       </c>
       <c r="F162">
@@ -2671,7 +2684,7 @@
       </c>
     </row>
     <row r="163" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B163" t="s">
+      <c r="B163" s="1" t="s">
         <v>85</v>
       </c>
       <c r="C163">
@@ -2680,7 +2693,7 @@
       <c r="D163">
         <v>9.8500000000000004E-2</v>
       </c>
-      <c r="E163">
+      <c r="E163" s="1">
         <v>2</v>
       </c>
       <c r="F163">
@@ -2688,7 +2701,7 @@
       </c>
     </row>
     <row r="164" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B164" t="s">
+      <c r="B164" s="1" t="s">
         <v>86</v>
       </c>
       <c r="C164">
@@ -2697,7 +2710,7 @@
       <c r="D164">
         <v>9.8500000000000004E-2</v>
       </c>
-      <c r="E164">
+      <c r="E164" s="1">
         <v>5</v>
       </c>
       <c r="F164">
@@ -2705,7 +2718,7 @@
       </c>
     </row>
     <row r="165" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B165" t="s">
+      <c r="B165" s="1" t="s">
         <v>87</v>
       </c>
       <c r="C165">
@@ -2714,7 +2727,7 @@
       <c r="D165">
         <v>9.8500000000000004E-2</v>
       </c>
-      <c r="E165">
+      <c r="E165" s="1">
         <v>4</v>
       </c>
       <c r="F165">
@@ -2722,7 +2735,7 @@
       </c>
     </row>
     <row r="166" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B166" t="s">
+      <c r="B166" s="1" t="s">
         <v>88</v>
       </c>
       <c r="C166">
@@ -2731,7 +2744,7 @@
       <c r="D166">
         <v>9.8500000000000004E-2</v>
       </c>
-      <c r="E166">
+      <c r="E166" s="1">
         <v>15</v>
       </c>
       <c r="F166">
@@ -2739,7 +2752,7 @@
       </c>
     </row>
     <row r="167" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B167" t="s">
+      <c r="B167" s="1" t="s">
         <v>89</v>
       </c>
       <c r="C167">
@@ -2748,7 +2761,7 @@
       <c r="D167">
         <v>9.8500000000000004E-2</v>
       </c>
-      <c r="E167">
+      <c r="E167" s="1">
         <v>2</v>
       </c>
       <c r="F167">
@@ -2756,7 +2769,7 @@
       </c>
     </row>
     <row r="168" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B168" t="s">
+      <c r="B168" s="1" t="s">
         <v>90</v>
       </c>
       <c r="C168">
@@ -2765,7 +2778,7 @@
       <c r="D168">
         <v>9.8500000000000004E-2</v>
       </c>
-      <c r="E168">
+      <c r="E168" s="1">
         <v>1</v>
       </c>
       <c r="F168">
@@ -2773,7 +2786,7 @@
       </c>
     </row>
     <row r="169" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B169" t="s">
+      <c r="B169" s="1" t="s">
         <v>60</v>
       </c>
       <c r="C169">
@@ -2782,7 +2795,7 @@
       <c r="D169">
         <v>9.8500000000000004E-2</v>
       </c>
-      <c r="E169">
+      <c r="E169" s="1">
         <v>2</v>
       </c>
       <c r="F169">
@@ -2790,7 +2803,7 @@
       </c>
     </row>
     <row r="170" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B170" t="s">
+      <c r="B170" s="1" t="s">
         <v>91</v>
       </c>
       <c r="C170">
@@ -2799,7 +2812,7 @@
       <c r="D170">
         <v>9.8500000000000004E-2</v>
       </c>
-      <c r="E170">
+      <c r="E170" s="1">
         <v>2</v>
       </c>
       <c r="F170">
@@ -2807,7 +2820,7 @@
       </c>
     </row>
     <row r="171" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B171" t="s">
+      <c r="B171" s="1" t="s">
         <v>61</v>
       </c>
       <c r="C171">
@@ -2816,7 +2829,7 @@
       <c r="D171">
         <v>9.8500000000000004E-2</v>
       </c>
-      <c r="E171">
+      <c r="E171" s="1">
         <v>4</v>
       </c>
       <c r="F171">
@@ -2824,7 +2837,7 @@
       </c>
     </row>
     <row r="172" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B172" t="s">
+      <c r="B172" s="1" t="s">
         <v>92</v>
       </c>
       <c r="C172">
@@ -2833,7 +2846,7 @@
       <c r="D172">
         <v>9.8500000000000004E-2</v>
       </c>
-      <c r="E172">
+      <c r="E172" s="1">
         <v>3</v>
       </c>
       <c r="F172">
@@ -2841,7 +2854,7 @@
       </c>
     </row>
     <row r="173" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B173" t="s">
+      <c r="B173" s="1" t="s">
         <v>93</v>
       </c>
       <c r="C173">
@@ -2850,7 +2863,7 @@
       <c r="D173">
         <v>9.8500000000000004E-2</v>
       </c>
-      <c r="E173">
+      <c r="E173" s="1">
         <v>2</v>
       </c>
       <c r="F173">
@@ -2858,7 +2871,7 @@
       </c>
     </row>
     <row r="174" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B174" t="s">
+      <c r="B174" s="1" t="s">
         <v>94</v>
       </c>
       <c r="C174">
@@ -2867,7 +2880,7 @@
       <c r="D174">
         <v>9.8500000000000004E-2</v>
       </c>
-      <c r="E174">
+      <c r="E174" s="1">
         <v>2</v>
       </c>
       <c r="F174">
@@ -2875,7 +2888,7 @@
       </c>
     </row>
     <row r="175" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B175" t="s">
+      <c r="B175" s="1" t="s">
         <v>95</v>
       </c>
       <c r="C175">
@@ -2884,7 +2897,7 @@
       <c r="D175">
         <v>9.8500000000000004E-2</v>
       </c>
-      <c r="E175">
+      <c r="E175" s="1">
         <v>3</v>
       </c>
       <c r="F175">
@@ -2892,7 +2905,7 @@
       </c>
     </row>
     <row r="176" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B176" t="s">
+      <c r="B176" s="1" t="s">
         <v>96</v>
       </c>
       <c r="C176">
@@ -2901,7 +2914,7 @@
       <c r="D176">
         <v>9.8500000000000004E-2</v>
       </c>
-      <c r="E176">
+      <c r="E176" s="1">
         <v>12</v>
       </c>
       <c r="F176">
@@ -2909,7 +2922,7 @@
       </c>
     </row>
     <row r="177" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B177" t="s">
+      <c r="B177" s="1" t="s">
         <v>97</v>
       </c>
       <c r="C177">
@@ -2918,7 +2931,7 @@
       <c r="D177">
         <v>9.8500000000000004E-2</v>
       </c>
-      <c r="E177">
+      <c r="E177" s="1">
         <v>2</v>
       </c>
       <c r="F177">
@@ -2926,7 +2939,7 @@
       </c>
     </row>
     <row r="178" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B178" t="s">
+      <c r="B178" s="1" t="s">
         <v>98</v>
       </c>
       <c r="C178">
@@ -2935,7 +2948,7 @@
       <c r="D178">
         <v>9.8500000000000004E-2</v>
       </c>
-      <c r="E178">
+      <c r="E178" s="1">
         <v>3</v>
       </c>
       <c r="F178">
@@ -2943,7 +2956,7 @@
       </c>
     </row>
     <row r="179" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B179" t="s">
+      <c r="B179" s="1" t="s">
         <v>99</v>
       </c>
       <c r="C179">
@@ -2952,7 +2965,7 @@
       <c r="D179">
         <v>9.8500000000000004E-2</v>
       </c>
-      <c r="E179">
+      <c r="E179" s="1">
         <v>3</v>
       </c>
       <c r="F179">
@@ -2960,7 +2973,7 @@
       </c>
     </row>
     <row r="180" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B180" t="s">
+      <c r="B180" s="1" t="s">
         <v>100</v>
       </c>
       <c r="C180">
@@ -2969,7 +2982,7 @@
       <c r="D180">
         <v>9.8500000000000004E-2</v>
       </c>
-      <c r="E180">
+      <c r="E180" s="1">
         <v>6</v>
       </c>
       <c r="F180">
@@ -2977,7 +2990,7 @@
       </c>
     </row>
     <row r="181" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B181" t="s">
+      <c r="B181" s="1" t="s">
         <v>101</v>
       </c>
       <c r="C181">
@@ -2986,7 +2999,7 @@
       <c r="D181">
         <v>9.8500000000000004E-2</v>
       </c>
-      <c r="E181">
+      <c r="E181" s="1">
         <v>2</v>
       </c>
       <c r="F181">
@@ -2994,7 +3007,7 @@
       </c>
     </row>
     <row r="182" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B182" t="s">
+      <c r="B182" s="1" t="s">
         <v>102</v>
       </c>
       <c r="C182">
@@ -3003,7 +3016,7 @@
       <c r="D182">
         <v>9.8500000000000004E-2</v>
       </c>
-      <c r="E182">
+      <c r="E182" s="1">
         <v>2</v>
       </c>
       <c r="F182">
@@ -3011,7 +3024,7 @@
       </c>
     </row>
     <row r="183" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B183" t="s">
+      <c r="B183" s="1" t="s">
         <v>103</v>
       </c>
       <c r="C183">
@@ -3020,7 +3033,7 @@
       <c r="D183">
         <v>9.8500000000000004E-2</v>
       </c>
-      <c r="E183">
+      <c r="E183" s="1">
         <v>9</v>
       </c>
       <c r="F183">
@@ -3028,7 +3041,7 @@
       </c>
     </row>
     <row r="184" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B184" t="s">
+      <c r="B184" s="1" t="s">
         <v>104</v>
       </c>
       <c r="C184">
@@ -3037,7 +3050,7 @@
       <c r="D184">
         <v>9.8500000000000004E-2</v>
       </c>
-      <c r="E184">
+      <c r="E184" s="1">
         <v>2</v>
       </c>
       <c r="F184">
@@ -3045,7 +3058,7 @@
       </c>
     </row>
     <row r="185" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B185" t="s">
+      <c r="B185" s="1" t="s">
         <v>105</v>
       </c>
       <c r="C185">
@@ -3054,7 +3067,7 @@
       <c r="D185">
         <v>9.8500000000000004E-2</v>
       </c>
-      <c r="E185">
+      <c r="E185" s="1">
         <v>2</v>
       </c>
       <c r="F185">
@@ -3070,7 +3083,7 @@
       </c>
     </row>
     <row r="189" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B189" t="s">
+      <c r="B189" s="1" t="s">
         <v>107</v>
       </c>
       <c r="C189">
@@ -3081,7 +3094,7 @@
       </c>
     </row>
     <row r="190" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B190" t="s">
+      <c r="B190" s="1" t="s">
         <v>108</v>
       </c>
       <c r="C190">
@@ -3092,7 +3105,7 @@
       </c>
     </row>
     <row r="191" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B191" t="s">
+      <c r="B191" s="1" t="s">
         <v>109</v>
       </c>
       <c r="C191">
@@ -3103,7 +3116,7 @@
       </c>
     </row>
     <row r="192" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B192" t="s">
+      <c r="B192" s="1" t="s">
         <v>110</v>
       </c>
       <c r="C192">
@@ -3114,7 +3127,7 @@
       </c>
     </row>
     <row r="193" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B193" t="s">
+      <c r="B193" s="1" t="s">
         <v>111</v>
       </c>
       <c r="C193">
@@ -3125,7 +3138,7 @@
       </c>
     </row>
     <row r="194" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B194" t="s">
+      <c r="B194" s="1" t="s">
         <v>60</v>
       </c>
       <c r="C194">
@@ -3141,7 +3154,7 @@
       </c>
     </row>
     <row r="198" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B198" t="s">
+      <c r="B198" s="1" t="s">
         <v>107</v>
       </c>
       <c r="C198">
@@ -3150,7 +3163,7 @@
       <c r="D198">
         <v>25.3202</v>
       </c>
-      <c r="E198">
+      <c r="E198" s="1">
         <v>836</v>
       </c>
       <c r="F198">
@@ -3158,7 +3171,7 @@
       </c>
     </row>
     <row r="199" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B199" t="s">
+      <c r="B199" s="1" t="s">
         <v>108</v>
       </c>
       <c r="C199">
@@ -3167,7 +3180,7 @@
       <c r="D199">
         <v>23.7438</v>
       </c>
-      <c r="E199">
+      <c r="E199" s="1">
         <v>861</v>
       </c>
       <c r="F199">
@@ -3175,7 +3188,7 @@
       </c>
     </row>
     <row r="200" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B200" t="s">
+      <c r="B200" s="1" t="s">
         <v>109</v>
       </c>
       <c r="C200">
@@ -3184,7 +3197,7 @@
       <c r="D200">
         <v>5.1231999999999998</v>
       </c>
-      <c r="E200">
+      <c r="E200" s="1">
         <v>138</v>
       </c>
       <c r="F200">
@@ -3192,7 +3205,7 @@
       </c>
     </row>
     <row r="201" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B201" t="s">
+      <c r="B201" s="1" t="s">
         <v>110</v>
       </c>
       <c r="C201">
@@ -3201,7 +3214,7 @@
       <c r="D201">
         <v>4.7290999999999999</v>
       </c>
-      <c r="E201">
+      <c r="E201" s="1">
         <v>186</v>
       </c>
       <c r="F201">
@@ -3209,7 +3222,7 @@
       </c>
     </row>
     <row r="202" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B202" t="s">
+      <c r="B202" s="1" t="s">
         <v>111</v>
       </c>
       <c r="C202">
@@ -3218,7 +3231,7 @@
       <c r="D202">
         <v>1.1822999999999999</v>
       </c>
-      <c r="E202">
+      <c r="E202" s="1">
         <v>23</v>
       </c>
       <c r="F202">
@@ -3226,7 +3239,7 @@
       </c>
     </row>
     <row r="203" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B203" t="s">
+      <c r="B203" s="1" t="s">
         <v>113</v>
       </c>
       <c r="C203">
@@ -3235,7 +3248,7 @@
       <c r="D203">
         <v>0.39410000000000001</v>
       </c>
-      <c r="E203">
+      <c r="E203" s="1">
         <v>13</v>
       </c>
       <c r="F203">
@@ -3243,7 +3256,7 @@
       </c>
     </row>
     <row r="204" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B204" t="s">
+      <c r="B204" s="1" t="s">
         <v>114</v>
       </c>
       <c r="C204">
@@ -3252,7 +3265,7 @@
       <c r="D204">
         <v>0.39410000000000001</v>
       </c>
-      <c r="E204">
+      <c r="E204" s="1">
         <v>13</v>
       </c>
       <c r="F204">
@@ -3260,7 +3273,7 @@
       </c>
     </row>
     <row r="205" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B205" t="s">
+      <c r="B205" s="1" t="s">
         <v>115</v>
       </c>
       <c r="C205">
@@ -3269,7 +3282,7 @@
       <c r="D205">
         <v>0.19700000000000001</v>
       </c>
-      <c r="E205">
+      <c r="E205" s="1">
         <v>4</v>
       </c>
       <c r="F205">
@@ -3277,7 +3290,7 @@
       </c>
     </row>
     <row r="206" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B206" t="s">
+      <c r="B206" s="1" t="s">
         <v>60</v>
       </c>
       <c r="C206">
@@ -3286,7 +3299,7 @@
       <c r="D206">
         <v>9.8500000000000004E-2</v>
       </c>
-      <c r="E206">
+      <c r="E206" s="1">
         <v>2</v>
       </c>
       <c r="F206">

</xml_diff>